<commit_message>
Add CMS articles Excel export; fill blog import tags and meta keywords
- Export Topics + Articles to .xlsx matching blog import column layout (cms/article.export)
- Add download link on Articles admin; en-gb/fr-fr text_export strings
- Populate meta_keyword and tag columns in shared/import/blog_import.xlsx

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/shared/import/blog_import.xlsx
+++ b/shared/import/blog_import.xlsx
@@ -661,7 +661,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -708,8 +707,16 @@
           <t>🤭До переїзду в місто у нас була можливість засаджувати великі площі овочевими культурами, і ми не особливо хвилювалися про віддачу, за рахунок багатьох грядок завжди мали достатньо продукції не тільки для себе, а й на продаж. Але з переїздом все змінилося, на десяти сотках багато не насадиш, і ми почали шукати нові мож</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>овочівництво, город, органічні овочі, насіння, поради городникам, дача</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>овочівництво, город, органіка, насіння, дача, поради</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>2020-05-19 19:55:28</t>
@@ -722,7 +729,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -769,8 +775,16 @@
           <t>🌶🥕🥑 Виходячи з того, що ми хочемо, чистіше, дешевше і смачніше при виборі сортів томатів все-таки намагаємося знайти стійкі до хвороб, змін погоди. Це найчастіше ранні та середні сорти, які встигають дозрівати до спекотної та вологої погоди. До них відносяться Дубок, Резонанс, Персей, Помаранчеве диво, Чайка, Волгоград</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>томати, сорти томатів, насіння томатів, вирощування томатів, салатні томати, гібриди</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>томати, сорти томатів, насіння, вирощування, біф-томати, ранні сорти</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>2020-05-19 22:04:52</t>
@@ -783,7 +797,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -830,8 +843,16 @@
           <t>🌶🥕🥑Огірок Китайське Чудо я спробувала посадити роки три тому, і не пошкодувала. Що б я не сідала надалі — йому завжди особливе місце. І хоча вважають, що головна відмінна риса цього сорту - дуже довгі плоди (40-60см), для мене - це ніжна м'якоть з надзвичайною хрустинкою, смак без найменшої гіркоти, незважаючи на погод</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>огірки, огірок китайське чудо, насіння огірків, вирощування огірків, теплиця</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>огірки, китайське чудо, насіння, вирощування, теплиця</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>2020-05-23 12:21:06</t>
@@ -844,7 +865,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -891,8 +911,16 @@
           <t>🌶🥕🥝СЕЛЕР. Купуючи фірмове насіння селери городники думають, що з їх вирощуванням немає жодних проблем, але не тут було! Замість великих їстівних коренеплодів чомусь виростають непоказні коріння майже як у листового селери. вегетативний період у селери дуже тривалий 150-180 днів залежно від сорту. І ось кілька секретів</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>селера, коренева селера, насіння селери, вирощування селери, розсада</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>селера, коренева селера, насіння, вирощування, посів, пікіровка</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>2020-06-03 00:16:10</t>
@@ -905,7 +933,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -952,8 +979,16 @@
           <t>🌶🥕🥝 На полях жнива, повним ходом йде збирання зернових, а у нас томати просять що б їм допомогли. В першу чергу правильне пасинкування звичайно наочно показати краще, але якщо ви зробите мінімально точно що написано буде. При пасинкуванні актуално не нашкодити тесть прибирати від землі 2-3 аркуша маючи на увазі що до б</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>томати, жнива, сезонні роботи, город, збір врожаю</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>томати, жнива, сезон, город, збір врожаю</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>2020-07-13 21:49:17</t>
@@ -966,7 +1001,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1013,8 +1047,16 @@
           <t>🌼 Пушкінія. Птахомлечник. Пушкінія та Птахомлечник цибулинні багаторічники, які довго не вимагають пересадки і ростуть на одному місці рясна цвітіння на третій рік після посадки. Належать до первоцвітів, тільки прогріється трохи земля, а вони бурхливо розростаються, викидаючи разом із щіткою зелені міцні квітконоси. Пе</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>пушкінія, птахомлечник, цибулинні квіти, клумба, ландшафт</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>пушкінія, птахомлечник, цибулинні, квіти, ландшафт</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>2020-07-25 22:12:15</t>
@@ -1027,7 +1069,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Порівняння сортів</t>
@@ -1074,8 +1115,16 @@
           <t>🌶🥕🥝Сорт Бліво-Синій туман. Сорт американського походження обросший легендами про його лікувальні властивості і взагалі синьо-плідним приділено багато місця як лікувальним із-за присутності в плодах антоціанів які дійсно мають властивості впливати на серцево-судинну, усуваючи утворення тромбів, при ожирінні якимось диво</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>томати, порівняння сортів, бліво-синій туман, насіння, гібриди</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>томати, порівняння сортів, бліво-синій туман, насіння</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>2020-08-11 15:20:42</t>
@@ -1088,7 +1137,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1135,8 +1183,16 @@
           <t>🤭 Старовинний спосіб зберігання часнику. Хоча часник і можна купити цілий рік у супермаркеті, свій часник з домашньої грядки набагато смачніший, але тоді виникає питання як його зберегти. Ще до винаходу холодильників часник заплітали в косу і підвішували в прохолодному місці на горищі, в льоху, в сінях, де він зберігав</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>часник, зберігання часнику, заготівлі, овочі, погріб</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>часник, зберігання, заготівлі, город, традиції</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>2020-09-09 20:29:06</t>
@@ -1149,7 +1205,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1196,8 +1251,16 @@
           <t>🌿Що можна посіяти у листопаді? Підзимові посіви – найпоширеніший спосіб отримати ранній та якісний урожай на наступний рік. Рослини, посіяні під зиму, більш стійкі до несприятливих погодних умов та хвороб, краще ростуть і раніше дозрівають. З овочів сіють насіння моркви, буряків, пастернаку, листової петрушки, кропу, ц</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>листопад, підзимовий посів, посів овочів, город, насіння</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>листопад, підзимовий посів, посів, насіння, город</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>2020-10-27 09:01:46</t>
@@ -1210,7 +1273,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -1257,8 +1319,16 @@
           <t>Безцінний огірок А ви знали, що звичайний огірок має вражаючі властивості? Огірок містить усі необхідні людині вітаміни: В1, В2, В3, В5, В6, З, фолієву кислоту, залізо, кальцій, фосфор, магній, калій, цинк. Набридло витирати запітніле дзеркало у ванній після душу? Перед прийняттям душа змастіть дзеркало кружальцем огір</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>огірок, користь огірків, овочі, здоров'я, город</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>огірок, користь, овочі, город, поради</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>2022-09-19 15:49:33</t>
@@ -1271,7 +1341,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -1318,8 +1387,16 @@
           <t>Секрети вирощування гороху Щоб збільшити врожай гороху, а також розтягнути період плодоношення, маківку прищипують, після чого горох пускає кілька бічних пагонів. Прищипку можна проводити будь-якої миті, навіть коли рослини ще зовсім маленькі, проте краще це робити вранці сонячного дня, щоб ранка встигла підсохнути і р</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>горох, вирощування гороху, агротехніка гороху, насіння гороху, врожай</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>горох, вирощування, агротехніка, насіння, врожай</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>2024-06-23 09:32:27</t>
@@ -1332,7 +1409,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1379,8 +1455,16 @@
           <t>Правила цвітіння Королівської пеларгонії та через які помилки вона не цвіте 🌺 ▪️1. Недотримання температурного режиму у зимовий період. Королівська пеларгонія взимку не знаходиться в стані повного спокою, рослина продовжує свій ріст і в цей період у нових пагонах, що ростуть, формуються квіткові нирки тільки в умовах п</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>пеларгонія, пеларгонія королівська, квіти на балконі, догляд за квітами</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>пеларгонія, королівська пеларгонія, квіти, догляд, цвітіння</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>2024-07-05 10:31:16</t>
@@ -1393,7 +1477,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -1440,8 +1523,16 @@
           <t>Μіні - конспект по томатам 🍅 📍Томат не любить: 1. Загущення 2. Πepeлив 3. Χолодне ґрунт, низькі температури 4. Βуcoку. вище 30 (відпадають зав'язі) 6. Надлишок азоту (жування) - багато навізу, селітри та ін. 7. Πолив за листом 8. Ηоспостереження лівообігу 📍Томат любить: 1. Πповітрювання (повітряні ванни) 2. Регулярний</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>томати, агротехніка томатів, помилки городника, вирощування, теплиця</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>томати, агротехніка, помилки, вирощування, теплиця</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>2024-07-07 09:31:53</t>
@@ -1454,7 +1545,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -1501,8 +1591,16 @@
           <t>Овочі, які варто посадити поруч один з одним. 1. Чудове тріо: кукурудза, горох і гарбуз. Секрет їхнього спільного вирощування знaли ще американські індіанці. Кукурудза дасть опору гороху, який насичує грунт азотом. А гарбуз у свою чергу не дає рости бур'янам. 2. Ще одне вдале поєднання: цибуля і морква. Цибуля рятує мо</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>сусідство культур, грядка, кукурудза, горох, гарбуз, спільні посадки</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>сусідство культур, грядка, кукурудза, горох, гарбуз</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>2024-07-19 21:04:37</t>
@@ -1515,7 +1613,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1562,8 +1659,16 @@
           <t>😊 ❤️ 😁 🩷 ❤️ 😊 😊 🩷 ❤️ 😊 ❤️ 🩷 ❤️ 🩷 😊 🌱 Висушила біля печі пахучий кріп, пам'ятаючи настанови старого Оглоблі. Міцні кругляші ріпи і редьки, засипані на льох, стануть малою підмогою довгої зими. Часом до неї приходили сумніви: вона погана господиня, треба було б запасти куди більше; у їх сім'ї буде дитя, а отже, і турбот</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>кріп, сушіння зелені, заготівлі, традиції, город</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>кріп, заготівлі, сушіння, традиції, дача</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>2024-08-28 12:30:21</t>
@@ -1576,7 +1681,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Покрокові інструкції (посів, пересадка, збір врожаю)</t>
@@ -1623,8 +1727,16 @@
           <t>Кульбаби Одна людина вирішила зробити гарний зелений лужок. Він дуже пишався тим, яка вона йому вийшла: рівна, красива і зелена. Якось він побачив, що серед зеленої трави зацвіли кульбаби. Це його розлютило. Він вирвав квіти руками. Але, згодом, кульбаби знову з'явилися. Вони маскувались під звичайною травою. І, як люд</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>кульбаба, газон, лужок, багаторічники, ландшафт</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>кульбаба, газон, лужок, багаторічники</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>2024-10-22 16:08:52</t>
@@ -1637,7 +1749,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Покрокові інструкції (посів, пересадка, збір врожаю)</t>
@@ -1684,8 +1795,16 @@
           <t>Вирішуємо проблеми глоксинії: частина 1 Глоксинії – витончені та яскраві квіти, але їхнє вирощування може супроводжуватися труднощами. Якщо знати основні проблеми та їх причини, можна уникнути неприємностей та насолоджуватися пишним цвітінням. 🌸 Основні проблеми при вирощуванні - Не утворюється бульба. Це трапляється,</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>глоксинія, кімнатні рослини, догляд за глоксинією, квіти</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>глоксинія, кімнатні квіти, догляд, хвороби рослин</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>2025-02-01 20:26:26</t>
@@ -1698,7 +1817,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1745,8 +1863,16 @@
           <t>🌳 Кора дерев: яскраві акценти зимового саду ❄️ Привіт всім! Продовжую ділитися порадами щодо створення зимового саду. Першу частину ви можете знайти тут. Зимовий сад — це не просто простір, це гармонія зимового ландшафту, де кожен елемент робить свій внесок у створення унікальної атмосфери. Ось деякі рослини, які особл</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>кора дерев, зимовий сад, декор саду, ландшафт, акценти</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>кора дерев, зимовий сад, декор, ландшафт</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>2025-02-25 10:56:14</t>
@@ -1759,7 +1885,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1806,8 +1931,16 @@
           <t>🌟 Тапіарні форми: прикраса, яка надихає цілий рік! ❄️ Всім привіт! Продовжую розповідь про створення зимового саду (частина 1, частина 2, частина 3). Тапіарні форми — це більше, ніж елементи ландшафтного дизайну. Вони перетворюють сад на витвір мистецтва, який тішить око і влітку, і взимку. Уявіть акуратні кулі, витонч</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>топіар, формування рослин, декоративний сад, садовий декор</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>топіар, формування, декоративний сад, ландшафт</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>2025-02-28 23:50:16</t>
@@ -1820,7 +1953,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Календар посадок (по місяцях)</t>
@@ -1867,8 +1999,16 @@
           <t>ПРИТЧА ПРО НАСІННЯ Одного разу жінці наснився сон, що за прилавком магазину стояв Господь Бог. - Господи! Це Ти? - Вигукнула вона з радістю. - Так, це Я, - відповів Бог. - А що в Тебе можна купити? - Запитала жінка. - У мене можна купити все, - пролунала відповідь. - У такому разі дай мені, будь ласка, здоров'я, щастя,</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>насіння, календар посадок, город, покупка насіння, дача</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>насіння, календар посадок, город, дача, поради</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>2025-04-17 16:08:33</t>
@@ -1881,7 +2021,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -1928,8 +2067,16 @@
           <t>🌐Інтернет останнім часом рясніє статтями про заборону вирощування шавлії. Квітникари стурбовані цією інформацією, але варто звернути увагу, що є безліч видів шавлії. ⛔️Хочу роз'яснити, що під заборону підпадає так звана шавлія провісників, вона ж шавлія наркотична( Сальвія дивінорум, від латів Salvia divinorum). 🌿Salvi</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>шавлія, вирощування шавлії, лікарські рослини, город, обмеження</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>шавлія, лікарські рослини, вирощування, город</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>2025-05-30 12:23:34</t>
@@ -1942,7 +2089,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -1989,8 +2135,16 @@
           <t>🌿 1. Як підготувати теплицю до посадок 1) Прибирання та дезінфекція Заберіть усі рослинні залишки, коріння, бур'яни. Промийте каркас та плівку/полікарбонат теплою водою із содою. Ґрунт можна пролити гарячим розчином марганцівки або мідним купоросом – це зменшує ризик хвороб. 2) Заміна або оновлення ґрунту Зніміть 5-7 с</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>теплиця, підготовка теплиці, дезінфекція, весняні посадки, город</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>теплиця, підготовка, дезінфекція, посадки, город</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>2025-11-18 11:24:10</t>
@@ -2003,7 +2157,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>Сезонні поради</t>
@@ -2050,8 +2203,16 @@
           <t>🧑‍🌾 1. Что такое посадочный материал и почему он важен Посадочный материал — это всё, из чего 📌 можно вырастить овощи, фрукты, цветы деревья это могут быть семена, клубни, саженцы для получения стабильных урожаев как правило используется отборная и качественная по всем параметрам культура. Если хотите попробовать нов</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>посадковий матеріал, саджанці, розсада, якість насіння, город</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>посадковий матеріал, саджанці, розсада, насіння, город</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>2025-12-17 15:14:09</t>
@@ -2064,7 +2225,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -2111,8 +2271,16 @@
           <t>🌞 Чому варто вибирати ранні та тепличні сорти овочів Вибір правильного посадкового матеріалу – це не просто данина моді, а реальна економія часу, праці та впевненість у стабільному врожаї. Особливо це важливо для умов короткого сезону чи вирощування у теплиці. 🟩 Основні переваги ранніх сортів ✅ Швидке дозрівання - урож</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>ранні сорти, теплиця, овочі, насіння, вирощування</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>ранні сорти, теплиця, овочі, насіння, вирощування</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>2025-12-24 22:55:11</t>
@@ -2125,7 +2293,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -2172,8 +2339,16 @@
           <t>Пост 1. Грунти та ґрунтосуміші для розсади: чому кислотність вирішує все 🌱 Багато проблем з розсадою починаються не з насіння і не з поливу, а з невідповідної кислотності ґрунту. Що таке кислотність (pH) і чому вона важлива pH показує, наскільки грунт кислий або лужний від pH залежить, чи засвоюються поживні речовини п</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>розсада, ґрунт, кислотність ґрунту, ph ґрунту, городник</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>розсада, ґрунт, кислотність, ph, город</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>2026-01-16 12:19:15</t>
@@ -2186,7 +2361,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -2233,8 +2407,16 @@
           <t>🍇 Грунт для садової чорниці: без компромісів Продовжуючи тему субстратів та ґрунтових сумішей, скажу головне: чорниця — культура строга до кислотності, і «що є під рукою» тут не працює. 🔹 Кислотність (pH): 3,5-4,8 - оптимальний діапазон. При pH вище 5 чорниці перестає засвоювати харчування, навіть якщо воно є у ґрунті.</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>чорниця, садова чорниця, ґрунт для чорниці, субстрат, кислота</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>чорниця, садова чорниця, ґрунт, субстрат, ягідні</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>2026-01-23 14:44:11</t>
@@ -2247,7 +2429,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -2294,8 +2475,16 @@
           <t>🌙. ПОГОДНИК 🌖 4–15 лютого — Місяць Місяць Це період, коли активність йде всередину — коріння отримує велику енергію, і виконуються добре всі кореневі та очищувальні роботи. Сприятливо для: ✔ Посіву насіння зелені та ранніх овочів (салат, шпинат, кріп, петрушка) ✔ Проріджування та розпушування ґрунту ✔ Видалення сухих с</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>місячний календар, погодник, лютий, посіви за місяцем, біодинаміка</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>місячний календар, погодник, лютий, посіви, город</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>2026-02-12 12:49:41</t>
@@ -2308,7 +2497,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>Покрокові інструкції (посів, пересадка, збір врожаю)</t>
@@ -2355,8 +2543,16 @@
           <t>Чорна ніжка - жах садівників, чорна ніжка це грибкові захворювання, яке виникає при надлишковому звільненні та нестачі світла. Захворюють сіянці дуже рано, найчастіше ще до появи першого листя., Сміттєва ніжка іноді викликає загибель значної кількості розсади, в окремих випадках врятувати вдається тільки поодинокі сіян</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>чорна ніжка, розсада, хвороби розсади, профілактика, фітофтора</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>чорна ніжка, розсада, хвороби, профілактика, город</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>2026-02-12 13:13:59</t>
@@ -2369,7 +2565,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -2416,8 +2611,16 @@
           <t>ГРУНТІ, ЯКІ КАТЕГОРИЧНО НЕ ПІДХОДЯТИ ДЛЯ РОЗСАДІ ❗️Це Земля прямо з міста "Розсада не має імунітету до мільйонів бактерий, грибків та личинок шкідників, що мешкають у міському ґрунті", – пояснює експерт. У такій землі часто присутнє насіння бур'янів, яке забирає світло та воду, а чорнозем швидко ущільнюється, пригнічую</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>розсада, ґрунт для розсади, помилки городника, міський ґрунт, город</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>розсада, ґрунт, помилки, город, субстрат</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>2026-02-12 13:17:26</t>
@@ -2430,7 +2633,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>Календар посадок (по місяцях)</t>
@@ -2477,8 +2679,16 @@
           <t>Народні орієнтири березня На Євдокію (14 березня) - якщо сонячно, буде рання весна. На Сороки (22 березня) — приліт птахів, час розпочинати активні посіви. Якщо березень сухий — чекай на багатий урожай овочів. перо, селера кореневої, редька, якщо ви ближче на південь. На спадаючому Місяці добре йдуть коренеплоди 3 бере</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>березень, народні прикмети, календар посадок, весна, город</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>березень, прикмети, календар посадок, весна, город</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>2026-02-28 09:39:29</t>
@@ -2491,7 +2701,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>Гіди по вирощуванню культур</t>
@@ -2538,8 +2747,16 @@
           <t>Поки наші томати міцніють у теплиці, саме час зайнятися тим, що любить прохолоду і ранню весну. 🌱 Що можна сіяти прямо в ґрунт: Щавель — холодостійкий, сходить при +3…+5°C. Петрушка - проростає повільно, тому сіємо раніше. Цибуля-батун - дає раннє перо, чудово зимує. Шпинат – не любить спеку, березень для нього ідеальн</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>холодостійкі культури, теплиця, томати, ранньовесняні посіви, город</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>холодостійкі культури, теплиця, томати, посіви, город</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr">
         <is>
           <t>2026-03-01 20:03:35</t>

</xml_diff>

<commit_message>
Blog: category tag carousel + sale products; PDP SEO fallbacks; import product_links
- Blog article: category carousel (parent+child paths) at top; home sale carousel below
- Category model: getCategoryPathString; product sale links include path like product cards
- Product page: meta fallbacks, image alt, lazy-load gallery; category meta_keyword fallback
- Blog import: column P product_links, shared/import path; export splits description + product_links
- blog_import.xlsx: product_links column; styles for blog carousels

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/shared/import/blog_import.xlsx
+++ b/shared/import/blog_import.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
@@ -663,6 +663,11 @@
       <c r="O1" s="0" t="inlineStr">
         <is>
           <t>seo_keyword</t>
+        </is>
+      </c>
+      <c r="P1" s="0" t="inlineStr">
+        <is>
+          <t>product_links</t>
         </is>
       </c>
     </row>
@@ -737,6 +742,13 @@
       <c r="O2" s="0" t="inlineStr">
         <is>
           <t>blog-post-2</t>
+        </is>
+      </c>
+      <c r="P2" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Насіння томату «Апельсин»
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати середньорослі — категорія
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Усі овочі</t>
         </is>
       </c>
     </row>
@@ -816,6 +828,12 @@
       <c r="O3" s="0" t="inlineStr">
         <is>
           <t>blog-post-6</t>
+        </is>
+      </c>
+      <c r="P3" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння овочів (огірки та ін.)
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -922,6 +940,12 @@
           <t>blog-post-11</t>
         </is>
       </c>
+      <c r="P4" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Зелень і овочі
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="n">
@@ -1006,6 +1030,12 @@
       <c r="O5" s="0" t="inlineStr">
         <is>
           <t>blog-post-32</t>
+        </is>
+      </c>
+      <c r="P5" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Томат «Апельсин»
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Насіння томатів</t>
         </is>
       </c>
     </row>
@@ -1093,6 +1123,12 @@
       <c r="O6" s="0" t="inlineStr">
         <is>
           <t>blog-post-38</t>
+        </is>
+      </c>
+      <c r="P6" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння квітів і овочів
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -1190,6 +1226,12 @@
       <c r="O7" s="0" t="inlineStr">
         <is>
           <t>blog-post-43</t>
+        </is>
+      </c>
+      <c r="P7" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Насіння томату «Апельсин»
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Сорти томатів</t>
         </is>
       </c>
     </row>
@@ -1457,6 +1499,12 @@
           <t>blog-post-52</t>
         </is>
       </c>
+      <c r="P8" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Посадковий матеріал і овочі
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="n">
@@ -1584,6 +1632,12 @@
           <t>blog-post-55</t>
         </is>
       </c>
+      <c r="P9" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння для посіву
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="n">
@@ -1674,6 +1728,12 @@
       <c r="O10" s="0" t="inlineStr">
         <is>
           <t>blog-post-78</t>
+        </is>
+      </c>
+      <c r="P10" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Бобові та овочі
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -1778,6 +1838,12 @@
       <c r="O11" s="0" t="inlineStr">
         <is>
           <t>blog-post-84</t>
+        </is>
+      </c>
+      <c r="P11" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння квітів і декору
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати для порівняння</t>
         </is>
       </c>
     </row>
@@ -1890,6 +1956,12 @@
           <t>blog-post-85</t>
         </is>
       </c>
+      <c r="P12" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Томат «Апельсин»
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Насіння томатів</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="n">
@@ -1994,6 +2066,12 @@
       <c r="O13" s="0" t="inlineStr">
         <is>
           <t>blog-post-89</t>
+        </is>
+      </c>
+      <c r="P13" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Сумісні культури — насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2080,6 +2158,12 @@
           <t>blog-post-119</t>
         </is>
       </c>
+      <c r="P14" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння та товари для квітів
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="n">
@@ -2156,6 +2240,12 @@
       <c r="O15" s="0" t="inlineStr">
         <is>
           <t>blog-post-139</t>
+        </is>
+      </c>
+      <c r="P15" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Декор і насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2237,6 +2327,12 @@
       <c r="O16" s="0" t="inlineStr">
         <is>
           <t>blog-post-189</t>
+        </is>
+      </c>
+      <c r="P16" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння в каталозі
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2350,6 +2446,12 @@
           <t>blog-post-334</t>
         </is>
       </c>
+      <c r="P17" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Теплиця та насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати для теплиці</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="n">
@@ -2458,6 +2560,12 @@
           <t>blog-post-339</t>
         </is>
       </c>
+      <c r="P18" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Якісне насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати та інші овочі</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="n">
@@ -2541,6 +2649,12 @@
           <t>blog-post-341</t>
         </is>
       </c>
+      <c r="P19" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння для теплиці
+https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Приклад: томат «Апельсин»</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="n">
@@ -2649,6 +2763,12 @@
           <t>blog-post-351</t>
         </is>
       </c>
+      <c r="P20" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Ґрунти та насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="n">
@@ -2748,6 +2868,12 @@
       <c r="O21" s="0" t="inlineStr">
         <is>
           <t>blog-post-353</t>
+        </is>
+      </c>
+      <c r="P21" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Ягідні культури та овочі
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2874,6 +3000,12 @@
           <t>blog-post-359</t>
         </is>
       </c>
+      <c r="P22" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння за сезоном
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="n">
@@ -2983,6 +3115,12 @@
           <t>blog-post-360</t>
         </is>
       </c>
+      <c r="P23" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Розсада та насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="n">
@@ -3088,6 +3226,12 @@
       <c r="O24" s="0" t="inlineStr">
         <is>
           <t>blog-post-361</t>
+        </is>
+      </c>
+      <c r="P24" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Ґрунт і насіння
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -3260,6 +3404,12 @@
           <t>blog-post-363</t>
         </is>
       </c>
+      <c r="P25" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння навесні
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="n">
@@ -3363,6 +3513,13 @@
       <c r="O26" s="0" t="inlineStr">
         <is>
           <t>blog-post-364</t>
+        </is>
+      </c>
+      <c r="P26" s="0" t="inlineStr">
+        <is>
+          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Томат «Апельсин»
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати
+https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Зелень та овочі</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Blog: links in description only, remove carousel and column P
Merge product_links into blog_import.xlsx column D as blog-in-body-catalog-links
paragraphs; drop product_links column. Import reads D only; export writes full
HTML to D without splitting. Remove article links carousel (controller,
template, languages) and related CSS; add light styles for in-body catalog links.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/shared/import/blog_import.xlsx
+++ b/shared/import/blog_import.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
@@ -663,11 +663,6 @@
       <c r="O1" s="0" t="inlineStr">
         <is>
           <t>seo_keyword</t>
-        </is>
-      </c>
-      <c r="P1" s="0" t="inlineStr">
-        <is>
-          <t>product_links</t>
         </is>
       </c>
     </row>
@@ -692,7 +687,7 @@
 &amp;lt;p data-end=&amp;quot;646&amp;quot; data-start=&amp;quot;334&amp;quot;&amp;gt;До таких сортів належать: Дубок, Резонанс, Персей, Оранжеве диво, Чайка, Волгоградський 323, Дамські пальчики. Вони дружно достигають і одночасно віддають урожай (за винятком Дамських пальчиків), але гарантовано забезпечать вас ранніми салатами. Усі ці сорти також добре підходять для засолювання та консервації.&amp;lt;/p&amp;gt;
 &amp;lt;p data-end=&amp;quot;993&amp;quot; data-start=&amp;quot;648&amp;quot;&amp;gt;Втім, ми ж хочемо не лише рано, а й багато. До врожайних сортів належать так звані біф-томати (їх ще називають біфштексними або салатними): Русский размер, Бичаче серце, Битюг, Корнеєвський рожевий, а також гібриди Граніт і Пінк Унікум. Вони великі, смачні, довго плодоносять і дають рясний урожай, але мають один недолік — недовго зберігаються.&amp;lt;/p&amp;gt;
 &amp;lt;p data-end=&amp;quot;1060&amp;quot; data-is-last-node=&amp;quot;&amp;quot; data-is-only-node=&amp;quot;&amp;quot; data-start=&amp;quot;995&amp;quot;&amp;gt;Різноманіття сортів безмежне, і кожен обирає те, що йому до душі.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/product&amp;amp;language=uk-ua&amp;amp;product_id=2&amp;amp;path=100_102"&gt;Насіння томату «Апельсин»&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати середньорослі — категорія&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Усі овочі&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
@@ -742,13 +737,6 @@
       <c r="O2" s="0" t="inlineStr">
         <is>
           <t>blog-post-2</t>
-        </is>
-      </c>
-      <c r="P2" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Насіння томату «Апельсин»
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати середньорослі — категорія
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Усі овочі</t>
         </is>
       </c>
     </row>
@@ -778,7 +766,7 @@
 	&amp;lt;li data-end=&amp;quot;809&amp;quot; data-section-id=&amp;quot;13207o9&amp;quot; data-start=&amp;quot;729&amp;quot;&amp;gt;Для консервації їх все одно нарізають шматочками, тож форма не має значення.&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
 &amp;lt;p data-end=&amp;quot;880&amp;quot; data-start=&amp;quot;811&amp;quot;&amp;gt;Ті, хто спробував ці огірочки,&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;877&amp;quot; data-start=&amp;quot;842&amp;quot;&amp;gt;більше не відмовляються від них&amp;lt;/strong&amp;gt;.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння овочів (огірки та ін.)&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
@@ -828,12 +816,6 @@
       <c r="O3" s="0" t="inlineStr">
         <is>
           <t>blog-post-6</t>
-        </is>
-      </c>
-      <c r="P3" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння овочів (огірки та ін.)
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -888,7 +870,7 @@
 &amp;lt;/ul&amp;gt;
 &amp;lt;hr data-end=&amp;quot;1135&amp;quot; data-start=&amp;quot;1132&amp;quot; /&amp;gt;
 &amp;lt;p data-end=&amp;quot;1226&amp;quot; data-start=&amp;quot;1137&amp;quot;&amp;gt;💡 Дотримуючись цих простих правил, можна отримати&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1223&amp;quot; data-start=&amp;quot;1188&amp;quot;&amp;gt;великий і якісний урожай селери&amp;lt;/strong&amp;gt;.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Зелень і овочі&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
@@ -938,12 +920,6 @@
       <c r="O4" s="0" t="inlineStr">
         <is>
           <t>blog-post-11</t>
-        </is>
-      </c>
-      <c r="P4" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Зелень і овочі
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -980,7 +956,7 @@
 &amp;lt;/ul&amp;gt;
 &amp;lt;hr data-end=&amp;quot;753&amp;quot; data-start=&amp;quot;750&amp;quot; /&amp;gt;
 &amp;lt;p data-end=&amp;quot;850&amp;quot; data-start=&amp;quot;755&amp;quot;&amp;gt;💡 Дотримуючись цих правил, томати будуть зав’язуватися і плодоносити&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;847&amp;quot; data-start=&amp;quot;825&amp;quot;&amp;gt;стабільно та рясно&amp;lt;/strong&amp;gt;.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/product&amp;amp;language=uk-ua&amp;amp;product_id=2&amp;amp;path=100_102"&gt;Томат «Апельсин»&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Насіння томатів&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
@@ -1030,12 +1006,6 @@
       <c r="O5" s="0" t="inlineStr">
         <is>
           <t>blog-post-32</t>
-        </is>
-      </c>
-      <c r="P5" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Томат «Апельсин»
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Насіння томатів</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1043,7 @@
 &amp;lt;ul data-end=&amp;quot;973&amp;quot; data-start=&amp;quot;870&amp;quot;&amp;gt;
 	&amp;lt;li data-end=&amp;quot;973&amp;quot; data-section-id=&amp;quot;11khncl&amp;quot; data-start=&amp;quot;870&amp;quot;&amp;gt;&amp;lt;strong data-end=&amp;quot;883&amp;quot; data-start=&amp;quot;872&amp;quot;&amp;gt;Зимівля&amp;lt;/strong&amp;gt;: цибулини прекрасно переносять зиму у ґрунті, тому пересадку можна проводити не щороку.&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння квітів і овочів&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -1123,12 +1093,6 @@
       <c r="O6" s="0" t="inlineStr">
         <is>
           <t>blog-post-38</t>
-        </is>
-      </c>
-      <c r="P6" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння квітів і овочів
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1140,7 @@
 	&amp;lt;/li&amp;gt;
 	&amp;lt;li data-end=&amp;quot;1063&amp;quot; data-section-id=&amp;quot;cvbs7v&amp;quot; data-start=&amp;quot;1010&amp;quot;&amp;gt;&amp;lt;strong data-end=&amp;quot;1028&amp;quot; data-start=&amp;quot;1012&amp;quot;&amp;gt;Особливість:&amp;lt;/strong&amp;gt;&amp;amp;nbsp;сорт вважається&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1060&amp;quot; data-start=&amp;quot;1045&amp;quot;&amp;gt;колекційним&amp;lt;/strong&amp;gt;.&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/product&amp;amp;language=uk-ua&amp;amp;product_id=2&amp;amp;path=100_102"&gt;Насіння томату «Апельсин»&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Сорти томатів&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -1226,12 +1190,6 @@
       <c r="O7" s="0" t="inlineStr">
         <is>
           <t>blog-post-43</t>
-        </is>
-      </c>
-      <c r="P7" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Насіння томату «Апельсин»
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Сорти томатів</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1209,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">&amp;lt;p&amp;gt;&amp;amp;nbsp;&amp;lt;/p&amp;gt;
+          <t>&amp;lt;p&amp;gt;&amp;amp;nbsp;&amp;lt;/p&amp;gt;
 &amp;lt;p&amp;gt;&amp;lt;meta charset=&amp;quot;UTF-8&amp;quot; /&amp;gt;&amp;lt;/p&amp;gt;
 &amp;lt;section data-scroll-anchor=&amp;quot;false&amp;quot; data-testid=&amp;quot;conversation-turn-1&amp;quot; data-turn=&amp;quot;user&amp;quot; data-turn-id=&amp;quot;7b3c3c99-acc3-4b13-b6b2-1d50b6447465&amp;quot; dir=&amp;quot;auto&amp;quot;&amp;gt;
 &amp;lt;p&amp;gt;переведи на укр та додай заголовок. я буду присилати декілька текстів&amp;lt;/p&amp;gt;
@@ -1447,7 +1405,7 @@
 &amp;lt;/section&amp;gt;
 &amp;lt;section data-scroll-anchor=&amp;quot;false&amp;quot; data-testid=&amp;quot;conversation-turn-16&amp;quot; data-turn=&amp;quot;assistant&amp;quot; data-turn-id=&amp;quot;request-WEB:3ae20428-d822-4870-a930-ebfd077d691d-7&amp;quot; dir=&amp;quot;auto&amp;quot;&amp;gt;
 &amp;lt;p data-end=&amp;quot;76&amp;quot; data-start=&amp;quot;0&amp;quot;&amp;gt;Ось український переклад із заголовком і структурованим поділом на пункти:&amp;lt;/p&amp;gt;
-&amp;lt;hr </t>
+&amp;lt;hr &lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Посадковий матеріал і овочі&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -1497,12 +1455,6 @@
       <c r="O8" s="0" t="inlineStr">
         <is>
           <t>blog-post-52</t>
-        </is>
-      </c>
-      <c r="P8" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Посадковий матеріал і овочі
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1532,7 @@
 	&amp;lt;li data-end=&amp;quot;1203&amp;quot; data-section-id=&amp;quot;ettulb&amp;quot; data-start=&amp;quot;1191&amp;quot;&amp;gt;Ехінацея&amp;lt;/li&amp;gt;
 	&amp;lt;li data-end=&amp;quot;1226&amp;quot; data-section-id=&amp;quot;1ihzdnb&amp;quot; data-start=&amp;quot;1204&amp;quot;&amp;gt;Ліатріс колосковий&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння для посіву&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -1630,12 +1582,6 @@
       <c r="O9" s="0" t="inlineStr">
         <is>
           <t>blog-post-55</t>
-        </is>
-      </c>
-      <c r="P9" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння для посіву
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1624,7 @@
 &amp;lt;/ul&amp;gt;
 &amp;lt;hr data-end=&amp;quot;880&amp;quot; data-start=&amp;quot;877&amp;quot; /&amp;gt;
 &amp;lt;p data-end=&amp;quot;965&amp;quot; data-start=&amp;quot;882&amp;quot;&amp;gt;💡 Такий підхід дозволяє отримати&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;952&amp;quot; data-start=&amp;quot;916&amp;quot;&amp;gt;рясний та тривалий урожай гороху&amp;lt;/strong&amp;gt;&amp;amp;nbsp;на грядці.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Бобові та овочі&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -1728,12 +1674,6 @@
       <c r="O10" s="0" t="inlineStr">
         <is>
           <t>blog-post-78</t>
-        </is>
-      </c>
-      <c r="P10" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Бобові та овочі
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1728,7 @@
 &amp;lt;/ul&amp;gt;
 &amp;lt;hr data-end=&amp;quot;1149&amp;quot; data-start=&amp;quot;1146&amp;quot; /&amp;gt;
 &amp;lt;p data-end=&amp;quot;1256&amp;quot; data-start=&amp;quot;1151&amp;quot;&amp;gt;💡 Дотримуючись цих правил, можна забезпечити&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1253&amp;quot; data-start=&amp;quot;1197&amp;quot;&amp;gt;багате та регулярне цвітіння Королівської пеларгонії&amp;lt;/strong&amp;gt;.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння квітів і декору&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати для порівняння&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -1838,12 +1778,6 @@
       <c r="O11" s="0" t="inlineStr">
         <is>
           <t>blog-post-84</t>
-        </is>
-      </c>
-      <c r="P11" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння квітів і декору
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати для порівняння</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1838,7 @@
 &amp;lt;/ol&amp;gt;
 &amp;lt;hr data-end=&amp;quot;988&amp;quot; data-start=&amp;quot;985&amp;quot; /&amp;gt;
 &amp;lt;p data-end=&amp;quot;1072&amp;quot; data-start=&amp;quot;990&amp;quot;&amp;gt;💡 Дотримуючись цих правил, томати будуть&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1069&amp;quot; data-start=&amp;quot;1032&amp;quot;&amp;gt;здоровими, врожайними та смачними&amp;lt;/strong&amp;gt;.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/product&amp;amp;language=uk-ua&amp;amp;product_id=2&amp;amp;path=100_102"&gt;Томат «Апельсин»&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Насіння томатів&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E12" s="0" t="inlineStr">
@@ -1954,12 +1888,6 @@
       <c r="O12" s="0" t="inlineStr">
         <is>
           <t>blog-post-85</t>
-        </is>
-      </c>
-      <c r="P12" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Томат «Апельсин»
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Насіння томатів</t>
         </is>
       </c>
     </row>
@@ -2016,7 +1944,7 @@
 &amp;lt;/ul&amp;gt;
 &amp;lt;hr data-end=&amp;quot;1039&amp;quot; data-start=&amp;quot;1036&amp;quot; /&amp;gt;
 &amp;lt;p data-end=&amp;quot;1161&amp;quot; data-start=&amp;quot;1041&amp;quot;&amp;gt;💡&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1055&amp;quot; data-start=&amp;quot;1044&amp;quot;&amp;gt;Порада:&amp;lt;/strong&amp;gt;&amp;amp;nbsp;правильне сусідство овочів підвищує врожайність, зменшує кількість шкідників і покращує смак продукції.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Сумісні культури — насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -2066,12 +1994,6 @@
       <c r="O13" s="0" t="inlineStr">
         <is>
           <t>blog-post-89</t>
-        </is>
-      </c>
-      <c r="P13" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Сумісні культури — насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2028,7 @@
 	&amp;lt;li data-end=&amp;quot;1221&amp;quot; data-section-id=&amp;quot;1mh294l&amp;quot; data-start=&amp;quot;1095&amp;quot;&amp;gt;&amp;lt;strong data-end=&amp;quot;1154&amp;quot; data-start=&amp;quot;1097&amp;quot;&amp;gt;Краї листя загинаються, квіти формуються неправильно.&amp;lt;/strong&amp;gt;&amp;amp;nbsp;Надмірна вологість ґрунту негативно впливає на розвиток рослини.&amp;lt;/li&amp;gt;
 	&amp;lt;li data-end=&amp;quot;1335&amp;quot; data-section-id=&amp;quot;1gsc7u5&amp;quot; data-start=&amp;quot;1223&amp;quot;&amp;gt;&amp;lt;strong data-end=&amp;quot;1255&amp;quot; data-start=&amp;quot;1225&amp;quot;&amp;gt;Гниють черешки та бруньки.&amp;lt;/strong&amp;gt;&amp;amp;nbsp;Винуватцем може бути занадто кислий ґрунт, надлишок азоту або переувлажнення.&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння та товари для квітів&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -2156,12 +2078,6 @@
       <c r="O14" s="0" t="inlineStr">
         <is>
           <t>blog-post-119</t>
-        </is>
-      </c>
-      <c r="P14" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння та товари для квітів
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2106,7 @@
 &amp;lt;p&amp;gt;➖ Пагони дерену — одні оливкового, інші червоно-оранжевого відтінку! Ці контрастні кольори додають зимовому саду весняних ноток, оживляючи його.&amp;lt;/p&amp;gt;
 &amp;lt;p&amp;gt;➖ Клен зеленокорий зі світло-сірою та зеленою корою також не може не тішити око 🍃&amp;lt;/p&amp;gt;
 &amp;lt;p&amp;gt;➖ А берези зі своїми чистими, ніби вимитими, стовбурами гармонійно зливаються з білим снігом.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Декор і насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -2240,12 +2156,6 @@
       <c r="O15" s="0" t="inlineStr">
         <is>
           <t>blog-post-139</t>
-        </is>
-      </c>
-      <c r="P15" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Декор і насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2187,7 @@
 Через деякий час він повернувся з маленькою паперовою коробочкою.&amp;lt;/p&amp;gt;
 &amp;lt;p&amp;gt;— І це все?! — вигукнула здивована й розчарована жінка.&amp;lt;br /&amp;gt;
 — Так, це все, — відповів Бог. — Хіба ти не знала, що в моєму магазині продається лише насіння?&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння в каталозі&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2327,12 +2237,6 @@
       <c r="O16" s="0" t="inlineStr">
         <is>
           <t>blog-post-189</t>
-        </is>
-      </c>
-      <c r="P16" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння в каталозі
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2298,7 @@
 Дуже швидкий продукт (7–12 днів).&amp;lt;br /&amp;gt;
 Особливо популярна перед святами для ресторанів і магазинів.&amp;lt;br /&amp;gt;
 Мінімальні витрати — максимальна маржинальність.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Теплиця та насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати для теплиці&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -2444,12 +2348,6 @@
       <c r="O17" s="0" t="inlineStr">
         <is>
           <t>blog-post-334</t>
-        </is>
-      </c>
-      <c r="P17" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Теплиця та насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати для теплиці</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2406,7 @@
 ✔ враховуйте норму висіву на 10–100 м²&amp;lt;/p&amp;gt;
 &amp;lt;h4 data-end=&amp;quot;2395&amp;quot; data-start=&amp;quot;2362&amp;quot;&amp;gt;📌 Облік терміну придатності&amp;lt;/h4&amp;gt;
 &amp;lt;p data-end=&amp;quot;2525&amp;quot; data-start=&amp;quot;2396&amp;quot;&amp;gt;Насіння втрачає схожість із часом, особливо дрібні трав’янисті види; своєчасна покупка та правильне зберігання — запорука успіху.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Якісне насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати та інші овочі&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -2558,12 +2456,6 @@
       <c r="O18" s="0" t="inlineStr">
         <is>
           <t>blog-post-339</t>
-        </is>
-      </c>
-      <c r="P18" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Якісне насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати та інші овочі</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2489,7 @@
 &amp;lt;p data-end=&amp;quot;1091&amp;quot; data-start=&amp;quot;989&amp;quot;&amp;gt;💡&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1014&amp;quot; data-start=&amp;quot;992&amp;quot;&amp;gt;Раннє плодоношення&amp;lt;/strong&amp;gt;&amp;amp;nbsp;— захищений ґрунт прискорює розвиток культури порівняно з відкритим полем.&amp;lt;/p&amp;gt;
 &amp;lt;p data-end=&amp;quot;1195&amp;quot; data-start=&amp;quot;1093&amp;quot;&amp;gt;🦠&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1113&amp;quot; data-start=&amp;quot;1096&amp;quot;&amp;gt;Менше стресів&amp;lt;/strong&amp;gt;&amp;amp;nbsp;— тепличні гібриди часто мають кращу стійкість до хвороб та коливань вологості.&amp;lt;/p&amp;gt;
 &amp;lt;p data-end=&amp;quot;1302&amp;quot; data-start=&amp;quot;1197&amp;quot;&amp;gt;🍅&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1230&amp;quot; data-start=&amp;quot;1200&amp;quot;&amp;gt;Більш стабільні результати&amp;lt;/strong&amp;gt;&amp;amp;nbsp;— особливо якщо це гібриди F1, які дають вирівняний і якісний урожай.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння для теплиці&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/product&amp;amp;language=uk-ua&amp;amp;product_id=2&amp;amp;path=100_102"&gt;Приклад: томат «Апельсин»&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -2647,12 +2539,6 @@
       <c r="O19" s="0" t="inlineStr">
         <is>
           <t>blog-post-341</t>
-        </is>
-      </c>
-      <c r="P19" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння для теплиці
-https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Приклад: томат «Апельсин»</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2597,7 @@
 &amp;lt;/ul&amp;gt;
 &amp;lt;p data-end=&amp;quot;1299&amp;quot; data-start=&amp;quot;1169&amp;quot;&amp;gt;💡 Важливо знати: дешеві торф’яні ґрунти часто бувають&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1241&amp;quot; data-start=&amp;quot;1224&amp;quot;&amp;gt;перекисленими&amp;lt;/strong&amp;gt;. Зовні вони пухкі та гарні, але розсада в них «стоить».&amp;lt;/p&amp;gt;
 &amp;lt;p data-end=&amp;quot;1403&amp;quot; data-start=&amp;quot;1301&amp;quot;&amp;gt;👉 В «Fun Dacha» — ґрунти з перевіреною кислотністю, підходять саме для вирощування здорової розсади.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Ґрунти та насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -2761,12 +2647,6 @@
       <c r="O20" s="0" t="inlineStr">
         <is>
           <t>blog-post-351</t>
-        </is>
-      </c>
-      <c r="P20" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Ґрунти та насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2698,7 @@
 	&amp;lt;li data-end=&amp;quot;883&amp;quot; data-section-id=&amp;quot;1gfqc1n&amp;quot; data-start=&amp;quot;856&amp;quot;&amp;gt;Хвоя, кора, кислий торф&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
 &amp;lt;p data-end=&amp;quot;994&amp;quot; data-start=&amp;quot;885&amp;quot;&amp;gt;Лохина росте повільно, але при правильному субстраті стабільно плодоносить&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;987&amp;quot; data-start=&amp;quot;960&amp;quot;&amp;gt;протягом багатьох років&amp;lt;/strong&amp;gt;&amp;amp;nbsp;🌱💚&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Ягідні культури та овочі&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -2868,12 +2748,6 @@
       <c r="O21" s="0" t="inlineStr">
         <is>
           <t>blog-post-353</t>
-        </is>
-      </c>
-      <c r="P21" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Ягідні культури та овочі
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2822,7 @@
 	&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
 &amp;lt;p data-end=&amp;quot;2282&amp;quot; data-start=&amp;quot;2201&amp;quot;&amp;gt;❗ Уникайте сильної обрізки дуже молодих дерев, щоб не травмувати кору в морози.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння за сезоном&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
@@ -2998,12 +2872,6 @@
       <c r="O22" s="0" t="inlineStr">
         <is>
           <t>blog-post-359</t>
-        </is>
-      </c>
-      <c r="P22" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння за сезоном
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -3063,7 +2931,7 @@
 	&amp;lt;/li&amp;gt;
 &amp;lt;/ol&amp;gt;
 &amp;lt;p data-end=&amp;quot;1328&amp;quot; data-start=&amp;quot;1203&amp;quot;&amp;gt;💡 Здається простим, але коли всі ці кроки зібрані в одному блоці, стає зрозуміло,&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;1325&amp;quot; data-start=&amp;quot;1286&amp;quot;&amp;gt;як правильно запобігти чорній ніжці&amp;lt;/strong&amp;gt;.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Розсада та насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -3113,12 +2981,6 @@
       <c r="O23" s="0" t="inlineStr">
         <is>
           <t>blog-post-360</t>
-        </is>
-      </c>
-      <c r="P23" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Розсада та насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3038,7 @@
 	&amp;lt;li data-end=&amp;quot;1584&amp;quot; data-section-id=&amp;quot;hngrnb&amp;quot; data-start=&amp;quot;1506&amp;quot;&amp;gt;Неприємні запахи (аміак, гниль, пліснява) свідчать про токсичність ґрунту.&amp;lt;/li&amp;gt;
 	&amp;lt;li data-end=&amp;quot;1662&amp;quot; data-section-id=&amp;quot;1fff0ui&amp;quot; data-start=&amp;quot;1585&amp;quot;&amp;gt;Наявність гілок, камінців або пластику — про низьку культуру виробництва.&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Ґрунт і насіння&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -3226,12 +3088,6 @@
       <c r="O24" s="0" t="inlineStr">
         <is>
           <t>blog-post-361</t>
-        </is>
-      </c>
-      <c r="P24" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Ґрунт і насіння
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3208,7 @@
 	&amp;lt;li data-end=&amp;quot;2186&amp;quot; data-section-id=&amp;quot;1rf37aq&amp;quot; data-start=&amp;quot;2112&amp;quot;&amp;gt;У березні&amp;amp;nbsp;&amp;lt;strong data-end=&amp;quot;2183&amp;quot; data-start=&amp;quot;2124&amp;quot;&amp;gt;не поспішайте з огірками та кабачками у відкритий ґрунт&amp;lt;/strong&amp;gt;.&amp;lt;/li&amp;gt;
 	&amp;lt;li data-end=&amp;quot;2247&amp;quot; data-section-id=&amp;quot;4ydorh&amp;quot; data-start=&amp;quot;2187&amp;quot;&amp;gt;Краще мати якісну, міцну розсаду, ніж витягнуті рослини.&amp;lt;/li&amp;gt;
 &amp;lt;/ul&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Насіння навесні&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -3402,12 +3258,6 @@
       <c r="O25" s="0" t="inlineStr">
         <is>
           <t>blog-post-363</t>
-        </is>
-      </c>
-      <c r="P25" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Насіння навесні
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3313,7 @@
 &amp;lt;hr data-end=&amp;quot;1343&amp;quot; data-start=&amp;quot;1340&amp;quot; /&amp;gt;
 &amp;lt;h4 data-end=&amp;quot;1369&amp;quot; data-start=&amp;quot;1345&amp;quot;&amp;gt;🌾 Хазяйський рада:&amp;lt;/h4&amp;gt;
 &amp;lt;p data-end=&amp;quot;1476&amp;quot; data-start=&amp;quot;1370&amp;quot;&amp;gt;Не поспішайте сіяти все одночасно. Робіть посіви з інтервалом 7–10 днів — зелень буде на столі постійно.&amp;lt;/p&amp;gt;
-&amp;lt;/div&amp;gt;</t>
+&amp;lt;/div&amp;gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/product&amp;amp;language=uk-ua&amp;amp;product_id=2&amp;amp;path=100_102"&gt;Томат «Апельсин»&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100_102"&gt;Томати&lt;/a&gt;&lt;/p&gt;&lt;p class="blog-in-body-catalog-links"&gt;&lt;a href="https://fun-dacha.com.ua/index.php?route=product/category&amp;amp;language=uk-ua&amp;amp;path=100"&gt;Зелень та овочі&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -3513,13 +3363,6 @@
       <c r="O26" s="0" t="inlineStr">
         <is>
           <t>blog-post-364</t>
-        </is>
-      </c>
-      <c r="P26" s="0" t="inlineStr">
-        <is>
-          <t>https://fun-dacha.com.ua/index.php?route=product/product&amp;language=uk-ua&amp;product_id=2&amp;path=100_102|Томат «Апельсин»
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100_102|Томати
-https://fun-dacha.com.ua/index.php?route=product/category&amp;language=uk-ua&amp;path=100|Зелень та овочі</t>
         </is>
       </c>
     </row>

</xml_diff>